<commit_message>
fix(catalog): remove duplicate Odawara entry and fix Omiya/Yomiuriland coordinates
</commit_message>
<xml_diff>
--- a/reports/manual_image_qa.xlsx
+++ b/reports/manual_image_qa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1835" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="841">
   <si>
     <t xml:space="preserve">Destination ID</t>
   </si>
@@ -1097,15 +1097,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://upload.wikimedia.org/wikipedia/commons/thumb/4/4a/Odaiba_close_up_-_2025_Jan_14_01-27PM.jpeg/3840px-Odaiba_close_up_-_2025_Jan_14_01-27PM.jpeg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">odawara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Odawara &amp; Manazuru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://upload.wikimedia.org/wikipedia/commons/thumb/3/38/Aerial_views_of_Odawara_Japan.jpg/250px-Aerial_views_of_Odawara_Japan.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">okuhida</t>
@@ -2753,7 +2744,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I262"/>
+  <dimension ref="A1:I261"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.39"/>
@@ -4878,10 +4869,10 @@
         <v>360</v>
       </c>
       <c r="E103" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F103" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G103" s="0" t="s">
         <v>361</v>
@@ -4898,10 +4889,10 @@
         <v>363</v>
       </c>
       <c r="E104" s="0" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F104" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G104" s="0" t="s">
         <v>364</v>
@@ -4918,7 +4909,7 @@
         <v>366</v>
       </c>
       <c r="E105" s="0" t="s">
-        <v>29</v>
+        <v>230</v>
       </c>
       <c r="F105" s="0" t="s">
         <v>30</v>
@@ -4938,10 +4929,10 @@
         <v>369</v>
       </c>
       <c r="E106" s="0" t="s">
-        <v>230</v>
+        <v>24</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G106" s="0" t="s">
         <v>370</v>
@@ -4958,10 +4949,10 @@
         <v>372</v>
       </c>
       <c r="E107" s="0" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="F107" s="0" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G107" s="0" t="s">
         <v>373</v>
@@ -4978,7 +4969,7 @@
         <v>375</v>
       </c>
       <c r="E108" s="0" t="s">
-        <v>146</v>
+        <v>29</v>
       </c>
       <c r="F108" s="0" t="s">
         <v>30</v>
@@ -4998,10 +4989,10 @@
         <v>378</v>
       </c>
       <c r="E109" s="0" t="s">
-        <v>29</v>
+        <v>124</v>
       </c>
       <c r="F109" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G109" s="0" t="s">
         <v>379</v>
@@ -5017,11 +5008,17 @@
       <c r="B110" s="0" t="s">
         <v>381</v>
       </c>
+      <c r="C110" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D110" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="E110" s="0" t="s">
-        <v>124</v>
+        <v>230</v>
       </c>
       <c r="F110" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G110" s="0" t="s">
         <v>382</v>
@@ -5037,12 +5034,6 @@
       <c r="B111" s="0" t="s">
         <v>384</v>
       </c>
-      <c r="C111" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D111" s="0" t="s">
-        <v>12</v>
-      </c>
       <c r="E111" s="0" t="s">
         <v>230</v>
       </c>
@@ -5064,7 +5055,7 @@
         <v>387</v>
       </c>
       <c r="E112" s="0" t="s">
-        <v>230</v>
+        <v>80</v>
       </c>
       <c r="F112" s="0" t="s">
         <v>30</v>
@@ -5084,7 +5075,7 @@
         <v>390</v>
       </c>
       <c r="E113" s="0" t="s">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="F113" s="0" t="s">
         <v>30</v>
@@ -5164,10 +5155,10 @@
         <v>402</v>
       </c>
       <c r="E117" s="0" t="s">
-        <v>29</v>
+        <v>263</v>
       </c>
       <c r="F117" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G117" s="0" t="s">
         <v>403</v>
@@ -5184,7 +5175,7 @@
         <v>405</v>
       </c>
       <c r="E118" s="0" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="F118" s="0" t="s">
         <v>14</v>
@@ -5204,7 +5195,7 @@
         <v>408</v>
       </c>
       <c r="E119" s="0" t="s">
-        <v>243</v>
+        <v>117</v>
       </c>
       <c r="F119" s="0" t="s">
         <v>14</v>
@@ -5224,10 +5215,10 @@
         <v>411</v>
       </c>
       <c r="E120" s="0" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="F120" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G120" s="0" t="s">
         <v>412</v>
@@ -5244,10 +5235,10 @@
         <v>414</v>
       </c>
       <c r="E121" s="0" t="s">
-        <v>29</v>
+        <v>124</v>
       </c>
       <c r="F121" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G121" s="0" t="s">
         <v>415</v>
@@ -5264,10 +5255,10 @@
         <v>417</v>
       </c>
       <c r="E122" s="0" t="s">
-        <v>124</v>
+        <v>29</v>
       </c>
       <c r="F122" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G122" s="0" t="s">
         <v>418</v>
@@ -5404,10 +5395,10 @@
         <v>438</v>
       </c>
       <c r="E129" s="0" t="s">
-        <v>29</v>
+        <v>263</v>
       </c>
       <c r="F129" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G129" s="0" t="s">
         <v>439</v>
@@ -5424,7 +5415,7 @@
         <v>441</v>
       </c>
       <c r="E130" s="0" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="F130" s="0" t="s">
         <v>14</v>
@@ -5444,10 +5435,10 @@
         <v>444</v>
       </c>
       <c r="E131" s="0" t="s">
-        <v>243</v>
+        <v>29</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G131" s="0" t="s">
         <v>445</v>
@@ -5464,7 +5455,7 @@
         <v>447</v>
       </c>
       <c r="E132" s="0" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="F132" s="0" t="s">
         <v>30</v>
@@ -5484,7 +5475,7 @@
         <v>450</v>
       </c>
       <c r="E133" s="0" t="s">
-        <v>62</v>
+        <v>234</v>
       </c>
       <c r="F133" s="0" t="s">
         <v>30</v>
@@ -5504,10 +5495,10 @@
         <v>453</v>
       </c>
       <c r="E134" s="0" t="s">
-        <v>234</v>
+        <v>293</v>
       </c>
       <c r="F134" s="0" t="s">
-        <v>30</v>
+        <v>251</v>
       </c>
       <c r="G134" s="0" t="s">
         <v>454</v>
@@ -5524,13 +5515,13 @@
         <v>456</v>
       </c>
       <c r="E135" s="0" t="s">
-        <v>293</v>
+        <v>117</v>
       </c>
       <c r="F135" s="0" t="s">
-        <v>251</v>
+        <v>14</v>
       </c>
       <c r="G135" s="0" t="s">
-        <v>457</v>
+        <v>169</v>
       </c>
       <c r="H135" s="0" t="s">
         <v>16</v>
@@ -5538,10 +5529,10 @@
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="0" t="s">
+        <v>457</v>
+      </c>
+      <c r="B136" s="0" t="s">
         <v>458</v>
-      </c>
-      <c r="B136" s="0" t="s">
-        <v>459</v>
       </c>
       <c r="E136" s="0" t="s">
         <v>117</v>
@@ -5550,7 +5541,7 @@
         <v>14</v>
       </c>
       <c r="G136" s="0" t="s">
-        <v>169</v>
+        <v>96</v>
       </c>
       <c r="H136" s="0" t="s">
         <v>16</v>
@@ -5558,10 +5549,10 @@
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="0" t="s">
+        <v>459</v>
+      </c>
+      <c r="B137" s="0" t="s">
         <v>460</v>
-      </c>
-      <c r="B137" s="0" t="s">
-        <v>461</v>
       </c>
       <c r="E137" s="0" t="s">
         <v>117</v>
@@ -5570,7 +5561,7 @@
         <v>14</v>
       </c>
       <c r="G137" s="0" t="s">
-        <v>96</v>
+        <v>461</v>
       </c>
       <c r="H137" s="0" t="s">
         <v>16</v>
@@ -5583,11 +5574,17 @@
       <c r="B138" s="0" t="s">
         <v>463</v>
       </c>
+      <c r="C138" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D138" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="E138" s="0" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
       <c r="F138" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G138" s="0" t="s">
         <v>464</v>
@@ -5603,12 +5600,6 @@
       <c r="B139" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="C139" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D139" s="0" t="s">
-        <v>12</v>
-      </c>
       <c r="E139" s="0" t="s">
         <v>35</v>
       </c>
@@ -5650,7 +5641,7 @@
         <v>472</v>
       </c>
       <c r="E141" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F141" s="0" t="s">
         <v>30</v>
@@ -5670,7 +5661,7 @@
         <v>475</v>
       </c>
       <c r="E142" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F142" s="0" t="s">
         <v>30</v>
@@ -5689,8 +5680,14 @@
       <c r="B143" s="0" t="s">
         <v>478</v>
       </c>
+      <c r="C143" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D143" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="E143" s="0" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F143" s="0" t="s">
         <v>30</v>
@@ -5722,7 +5719,7 @@
         <v>30</v>
       </c>
       <c r="G144" s="0" t="s">
-        <v>482</v>
+        <v>143</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>16</v>
@@ -5730,10 +5727,10 @@
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="0" t="s">
+        <v>482</v>
+      </c>
+      <c r="B145" s="0" t="s">
         <v>483</v>
-      </c>
-      <c r="B145" s="0" t="s">
-        <v>484</v>
       </c>
       <c r="C145" s="0" t="s">
         <v>28</v>
@@ -5748,7 +5745,7 @@
         <v>30</v>
       </c>
       <c r="G145" s="0" t="s">
-        <v>143</v>
+        <v>484</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>16</v>
@@ -5852,7 +5849,7 @@
         <v>30</v>
       </c>
       <c r="G149" s="0" t="s">
-        <v>496</v>
+        <v>430</v>
       </c>
       <c r="H149" s="0" t="s">
         <v>16</v>
@@ -5860,10 +5857,10 @@
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="0" t="s">
+        <v>496</v>
+      </c>
+      <c r="B150" s="0" t="s">
         <v>497</v>
-      </c>
-      <c r="B150" s="0" t="s">
-        <v>498</v>
       </c>
       <c r="C150" s="0" t="s">
         <v>28</v>
@@ -5878,7 +5875,7 @@
         <v>30</v>
       </c>
       <c r="G150" s="0" t="s">
-        <v>433</v>
+        <v>498</v>
       </c>
       <c r="H150" s="0" t="s">
         <v>16</v>
@@ -6256,13 +6253,13 @@
         <v>542</v>
       </c>
       <c r="C165" s="0" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D165" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E165" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F165" s="0" t="s">
         <v>30</v>
@@ -6444,7 +6441,7 @@
         <v>12</v>
       </c>
       <c r="E172" s="0" t="s">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="F172" s="0" t="s">
         <v>30</v>
@@ -6574,7 +6571,7 @@
         <v>12</v>
       </c>
       <c r="E177" s="0" t="s">
-        <v>80</v>
+        <v>230</v>
       </c>
       <c r="F177" s="0" t="s">
         <v>30</v>
@@ -6678,7 +6675,7 @@
         <v>12</v>
       </c>
       <c r="E181" s="0" t="s">
-        <v>230</v>
+        <v>62</v>
       </c>
       <c r="F181" s="0" t="s">
         <v>30</v>
@@ -6730,7 +6727,7 @@
         <v>12</v>
       </c>
       <c r="E183" s="0" t="s">
-        <v>62</v>
+        <v>234</v>
       </c>
       <c r="F183" s="0" t="s">
         <v>30</v>
@@ -6776,13 +6773,13 @@
         <v>602</v>
       </c>
       <c r="C185" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D185" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E185" s="0" t="s">
-        <v>234</v>
+        <v>146</v>
       </c>
       <c r="F185" s="0" t="s">
         <v>30</v>
@@ -6828,16 +6825,16 @@
         <v>608</v>
       </c>
       <c r="C187" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D187" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E187" s="0" t="s">
-        <v>146</v>
+        <v>13</v>
       </c>
       <c r="F187" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G187" s="0" t="s">
         <v>609</v>
@@ -6912,7 +6909,7 @@
         <v>12</v>
       </c>
       <c r="E190" s="0" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F190" s="0" t="s">
         <v>14</v>
@@ -6990,7 +6987,7 @@
         <v>12</v>
       </c>
       <c r="E193" s="0" t="s">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="F193" s="0" t="s">
         <v>14</v>
@@ -7172,7 +7169,7 @@
         <v>12</v>
       </c>
       <c r="E200" s="0" t="s">
-        <v>203</v>
+        <v>117</v>
       </c>
       <c r="F200" s="0" t="s">
         <v>14</v>
@@ -7192,7 +7189,7 @@
         <v>650</v>
       </c>
       <c r="C201" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D201" s="0" t="s">
         <v>12</v>
@@ -7218,13 +7215,13 @@
         <v>653</v>
       </c>
       <c r="C202" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D202" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E202" s="0" t="s">
-        <v>117</v>
+        <v>243</v>
       </c>
       <c r="F202" s="0" t="s">
         <v>14</v>
@@ -7244,7 +7241,7 @@
         <v>656</v>
       </c>
       <c r="C203" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D203" s="0" t="s">
         <v>12</v>
@@ -7270,7 +7267,7 @@
         <v>659</v>
       </c>
       <c r="C204" s="0" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D204" s="0" t="s">
         <v>12</v>
@@ -7296,16 +7293,16 @@
         <v>662</v>
       </c>
       <c r="C205" s="0" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D205" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E205" s="0" t="s">
-        <v>243</v>
+        <v>19</v>
       </c>
       <c r="F205" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G205" s="0" t="s">
         <v>663</v>
@@ -7354,7 +7351,7 @@
         <v>12</v>
       </c>
       <c r="E207" s="0" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F207" s="0" t="s">
         <v>20</v>
@@ -7380,7 +7377,7 @@
         <v>12</v>
       </c>
       <c r="E208" s="0" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="F208" s="0" t="s">
         <v>20</v>
@@ -7432,7 +7429,7 @@
         <v>12</v>
       </c>
       <c r="E210" s="0" t="s">
-        <v>58</v>
+        <v>317</v>
       </c>
       <c r="F210" s="0" t="s">
         <v>20</v>
@@ -7452,7 +7449,7 @@
         <v>680</v>
       </c>
       <c r="C211" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D211" s="0" t="s">
         <v>12</v>
@@ -7478,13 +7475,13 @@
         <v>683</v>
       </c>
       <c r="C212" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D212" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E212" s="0" t="s">
-        <v>317</v>
+        <v>172</v>
       </c>
       <c r="F212" s="0" t="s">
         <v>20</v>
@@ -7536,7 +7533,7 @@
         <v>12</v>
       </c>
       <c r="E214" s="0" t="s">
-        <v>172</v>
+        <v>321</v>
       </c>
       <c r="F214" s="0" t="s">
         <v>20</v>
@@ -7556,7 +7553,7 @@
         <v>692</v>
       </c>
       <c r="C215" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D215" s="0" t="s">
         <v>12</v>
@@ -7608,16 +7605,16 @@
         <v>698</v>
       </c>
       <c r="C217" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D217" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E217" s="0" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="F217" s="0" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="G217" s="0" t="s">
         <v>699</v>
@@ -7692,7 +7689,7 @@
         <v>12</v>
       </c>
       <c r="E220" s="0" t="s">
-        <v>303</v>
+        <v>75</v>
       </c>
       <c r="F220" s="0" t="s">
         <v>76</v>
@@ -7744,7 +7741,7 @@
         <v>12</v>
       </c>
       <c r="E222" s="0" t="s">
-        <v>75</v>
+        <v>207</v>
       </c>
       <c r="F222" s="0" t="s">
         <v>76</v>
@@ -7796,13 +7793,13 @@
         <v>12</v>
       </c>
       <c r="E224" s="0" t="s">
-        <v>207</v>
+        <v>720</v>
       </c>
       <c r="F224" s="0" t="s">
         <v>76</v>
       </c>
       <c r="G224" s="0" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="H224" s="0" t="s">
         <v>16</v>
@@ -7810,10 +7807,10 @@
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="0" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B225" s="0" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C225" s="0" t="s">
         <v>11</v>
@@ -7822,13 +7819,13 @@
         <v>12</v>
       </c>
       <c r="E225" s="0" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="F225" s="0" t="s">
         <v>76</v>
       </c>
       <c r="G225" s="0" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="H225" s="0" t="s">
         <v>16</v>
@@ -7836,10 +7833,10 @@
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="0" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B226" s="0" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C226" s="0" t="s">
         <v>11</v>
@@ -7848,10 +7845,10 @@
         <v>12</v>
       </c>
       <c r="E226" s="0" t="s">
-        <v>727</v>
+        <v>279</v>
       </c>
       <c r="F226" s="0" t="s">
-        <v>76</v>
+        <v>251</v>
       </c>
       <c r="G226" s="0" t="s">
         <v>728</v>
@@ -7874,7 +7871,7 @@
         <v>12</v>
       </c>
       <c r="E227" s="0" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="F227" s="0" t="s">
         <v>251</v>
@@ -7900,7 +7897,7 @@
         <v>12</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>293</v>
+        <v>250</v>
       </c>
       <c r="F228" s="0" t="s">
         <v>251</v>
@@ -7926,13 +7923,13 @@
         <v>12</v>
       </c>
       <c r="E229" s="0" t="s">
-        <v>250</v>
+        <v>737</v>
       </c>
       <c r="F229" s="0" t="s">
         <v>251</v>
       </c>
       <c r="G229" s="0" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="H229" s="0" t="s">
         <v>16</v>
@@ -7940,10 +7937,10 @@
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="0" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B230" s="0" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C230" s="0" t="s">
         <v>11</v>
@@ -7952,7 +7949,7 @@
         <v>12</v>
       </c>
       <c r="E230" s="0" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="F230" s="0" t="s">
         <v>251</v>
@@ -7978,13 +7975,13 @@
         <v>12</v>
       </c>
       <c r="E231" s="0" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="F231" s="0" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="G231" s="0" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="H231" s="0" t="s">
         <v>16</v>
@@ -7992,10 +7989,10 @@
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="0" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B232" s="0" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C232" s="0" t="s">
         <v>11</v>
@@ -8004,7 +8001,7 @@
         <v>12</v>
       </c>
       <c r="E232" s="0" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="F232" s="0" t="s">
         <v>259</v>
@@ -8030,7 +8027,7 @@
         <v>12</v>
       </c>
       <c r="E233" s="0" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="F233" s="0" t="s">
         <v>259</v>
@@ -8056,7 +8053,7 @@
         <v>12</v>
       </c>
       <c r="E234" s="0" t="s">
-        <v>747</v>
+        <v>313</v>
       </c>
       <c r="F234" s="0" t="s">
         <v>259</v>
@@ -8082,7 +8079,7 @@
         <v>12</v>
       </c>
       <c r="E235" s="0" t="s">
-        <v>313</v>
+        <v>258</v>
       </c>
       <c r="F235" s="0" t="s">
         <v>259</v>
@@ -8134,13 +8131,13 @@
         <v>12</v>
       </c>
       <c r="E237" s="0" t="s">
-        <v>258</v>
+        <v>763</v>
       </c>
       <c r="F237" s="0" t="s">
         <v>259</v>
       </c>
       <c r="G237" s="0" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="H237" s="0" t="s">
         <v>16</v>
@@ -8148,10 +8145,10 @@
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="0" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B238" s="0" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C238" s="0" t="s">
         <v>11</v>
@@ -8160,7 +8157,7 @@
         <v>12</v>
       </c>
       <c r="E238" s="0" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="F238" s="0" t="s">
         <v>259</v>
@@ -8186,13 +8183,13 @@
         <v>12</v>
       </c>
       <c r="E239" s="0" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="F239" s="0" t="s">
         <v>259</v>
       </c>
       <c r="G239" s="0" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="H239" s="0" t="s">
         <v>16</v>
@@ -8200,19 +8197,19 @@
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="0" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B240" s="0" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C240" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D240" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E240" s="0" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="F240" s="0" t="s">
         <v>259</v>
@@ -8232,19 +8229,19 @@
         <v>776</v>
       </c>
       <c r="C241" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D241" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E241" s="0" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="F241" s="0" t="s">
         <v>259</v>
       </c>
       <c r="G241" s="0" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="H241" s="0" t="s">
         <v>16</v>
@@ -8252,19 +8249,19 @@
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="0" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B242" s="0" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="C242" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D242" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E242" s="0" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="F242" s="0" t="s">
         <v>259</v>
@@ -8284,16 +8281,16 @@
         <v>783</v>
       </c>
       <c r="C243" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D243" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E243" s="0" t="s">
-        <v>780</v>
+        <v>162</v>
       </c>
       <c r="F243" s="0" t="s">
-        <v>259</v>
+        <v>162</v>
       </c>
       <c r="G243" s="0" t="s">
         <v>784</v>
@@ -8414,7 +8411,7 @@
         <v>798</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D248" s="0" t="s">
         <v>12</v>
@@ -8466,7 +8463,7 @@
         <v>804</v>
       </c>
       <c r="C250" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D250" s="0" t="s">
         <v>12</v>
@@ -8524,13 +8521,13 @@
         <v>12</v>
       </c>
       <c r="E252" s="0" t="s">
-        <v>162</v>
+        <v>811</v>
       </c>
       <c r="F252" s="0" t="s">
-        <v>162</v>
+        <v>811</v>
       </c>
       <c r="G252" s="0" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="H252" s="0" t="s">
         <v>16</v>
@@ -8538,10 +8535,10 @@
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="0" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B253" s="0" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C253" s="0" t="s">
         <v>11</v>
@@ -8550,10 +8547,10 @@
         <v>12</v>
       </c>
       <c r="E253" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F253" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="G253" s="0" t="s">
         <v>815</v>
@@ -8570,16 +8567,16 @@
         <v>817</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D254" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E254" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F254" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="G254" s="0" t="s">
         <v>818</v>
@@ -8596,16 +8593,16 @@
         <v>820</v>
       </c>
       <c r="C255" s="0" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D255" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E255" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F255" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="G255" s="0" t="s">
         <v>821</v>
@@ -8628,10 +8625,10 @@
         <v>12</v>
       </c>
       <c r="E256" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="F256" s="0" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="G256" s="0" t="s">
         <v>824</v>
@@ -8648,19 +8645,19 @@
         <v>826</v>
       </c>
       <c r="C257" s="0" t="s">
-        <v>11</v>
+        <v>827</v>
       </c>
       <c r="D257" s="0" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="E257" s="0" t="s">
-        <v>814</v>
+        <v>13</v>
       </c>
       <c r="F257" s="0" t="s">
-        <v>814</v>
+        <v>14</v>
       </c>
       <c r="G257" s="0" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="H257" s="0" t="s">
         <v>16</v>
@@ -8668,22 +8665,22 @@
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="0" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B258" s="0" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C258" s="0" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="D258" s="0" t="s">
         <v>45</v>
       </c>
       <c r="E258" s="0" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F258" s="0" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G258" s="0" t="s">
         <v>831</v>
@@ -8700,19 +8697,19 @@
         <v>833</v>
       </c>
       <c r="C259" s="0" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="D259" s="0" t="s">
         <v>45</v>
       </c>
       <c r="E259" s="0" t="s">
-        <v>29</v>
+        <v>234</v>
       </c>
       <c r="F259" s="0" t="s">
         <v>30</v>
       </c>
       <c r="G259" s="0" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="H259" s="0" t="s">
         <v>16</v>
@@ -8720,22 +8717,22 @@
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="0" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B260" s="0" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="C260" s="0" t="s">
-        <v>837</v>
+        <v>827</v>
       </c>
       <c r="D260" s="0" t="s">
         <v>45</v>
       </c>
       <c r="E260" s="0" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="F260" s="0" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G260" s="0" t="s">
         <v>838</v>
@@ -8752,47 +8749,21 @@
         <v>840</v>
       </c>
       <c r="C261" s="0" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="D261" s="0" t="s">
         <v>45</v>
       </c>
       <c r="E261" s="0" t="s">
-        <v>243</v>
+        <v>13</v>
       </c>
       <c r="F261" s="0" t="s">
         <v>14</v>
       </c>
       <c r="G261" s="0" t="s">
-        <v>841</v>
+        <v>609</v>
       </c>
       <c r="H261" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A262" s="0" t="s">
-        <v>842</v>
-      </c>
-      <c r="B262" s="0" t="s">
-        <v>843</v>
-      </c>
-      <c r="C262" s="0" t="s">
-        <v>830</v>
-      </c>
-      <c r="D262" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="E262" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F262" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G262" s="0" t="s">
-        <v>612</v>
-      </c>
-      <c r="H262" s="0" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>